<commit_message>
Add Kobo What3Words field integration
</commit_message>
<xml_diff>
--- a/forms/wwm_kobo_updated.xlsx
+++ b/forms/wwm_kobo_updated.xlsx
@@ -1,438 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="133">
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>label::English (en) (english (en))</t>
-  </si>
-  <si>
-    <t>hint::English (en) (english (en))</t>
-  </si>
-  <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>guidance_hint</t>
-  </si>
-  <si>
-    <t>appearance</t>
-  </si>
-  <si>
-    <t>relevant</t>
-  </si>
-  <si>
-    <t>constraint</t>
-  </si>
-  <si>
-    <t>parameters</t>
-  </si>
-  <si>
-    <t>calculation</t>
-  </si>
-  <si>
-    <t>start</t>
-  </si>
-  <si>
-    <t>end</t>
-  </si>
-  <si>
-    <t>today</t>
-  </si>
-  <si>
-    <t>begin_group</t>
-  </si>
-  <si>
-    <t>group_ih2au74</t>
-  </si>
-  <si>
-    <t>Section 1 – General Information</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>text</t>
-  </si>
-  <si>
-    <t>collector_name</t>
-  </si>
-  <si>
-    <t>Collector name</t>
-  </si>
-  <si>
-    <t>Name of the person collecting the sample.</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Philipp Schiffer</t>
-  </si>
-  <si>
-    <t>select_multiple iq6nb08</t>
-  </si>
-  <si>
-    <t>affiliation</t>
-  </si>
-  <si>
-    <t>Affiliation (research group / institute)</t>
-  </si>
-  <si>
-    <t>Enter the research group, laboratory, institute, or consortium responsible for this sampling. Use the official name.</t>
-  </si>
-  <si>
-    <t>minimal</t>
-  </si>
-  <si>
-    <t>affiliation_other</t>
-  </si>
-  <si>
-    <t>If "Other", please type the affiliation name</t>
-  </si>
-  <si>
-    <t>selected(${affiliation}, 'other')</t>
-  </si>
-  <si>
-    <t>. = ''</t>
-  </si>
-  <si>
-    <t>sample_id</t>
-  </si>
-  <si>
-    <t>Sample ID</t>
-  </si>
-  <si>
-    <t>Unique code for each sampling site. Use the format COUNTRY-YEAR-### (e.g., COL-2025-001).</t>
-  </si>
-  <si>
-    <t>COL-2025-001</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>sampling_date</t>
-  </si>
-  <si>
-    <t>Sampling Date</t>
-  </si>
-  <si>
-    <t>Date when the sample was taken.</t>
-  </si>
-  <si>
-    <t>2025-09-12</t>
-  </si>
-  <si>
-    <t>select_one cl7yy10</t>
-  </si>
-  <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>Country where the sample was collected.</t>
-  </si>
-  <si>
-    <t>Colombia</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>Notes / Comments</t>
-  </si>
-  <si>
-    <t>Any relevant observations.</t>
-  </si>
-  <si>
-    <t>“Moist soil near coffee plantation.”</t>
-  </si>
-  <si>
-    <t>multiline</t>
-  </si>
-  <si>
-    <t>end_group</t>
-  </si>
-  <si>
-    <t>group_kw39a24</t>
-  </si>
-  <si>
-    <t>Section 2 – Geolocation</t>
-  </si>
-  <si>
-    <t>geopoint</t>
-  </si>
-  <si>
-    <t>gps_coordinates</t>
-  </si>
-  <si>
-    <t>Sampling location</t>
-  </si>
-  <si>
-    <t>Record precise coordinates using the map or GPS device.</t>
-  </si>
-  <si>
-    <t>(captured automatically)</t>
-  </si>
-  <si>
-    <t>maps</t>
-  </si>
-  <si>
-    <t>site_name</t>
-  </si>
-  <si>
-    <t>Site name</t>
-  </si>
-  <si>
-    <t>Name or code for the sampling site.</t>
-  </si>
-  <si>
-    <t>“San Pedro plot”</t>
-  </si>
-  <si>
-    <t>group_jy8zq69</t>
-  </si>
-  <si>
-    <t>Section 3 – Environmental &amp; Soil Data</t>
-  </si>
-  <si>
-    <t>select_one ic4vv27</t>
-  </si>
-  <si>
-    <t>habitat_type</t>
-  </si>
-  <si>
-    <t>Habitat type</t>
-  </si>
-  <si>
-    <t>Select habitat (forest, agricultural, desert, grassland, etc.)</t>
-  </si>
-  <si>
-    <t>Agricultural field</t>
-  </si>
-  <si>
-    <t>select_one pt7uh58</t>
-  </si>
-  <si>
-    <t>soil_type</t>
-  </si>
-  <si>
-    <t>Soil type</t>
-  </si>
-  <si>
-    <t>Choose soil texture (sandy, clay, loamy, etc.)</t>
-  </si>
-  <si>
-    <t>Sandy loam</t>
-  </si>
-  <si>
-    <t>decimal</t>
-  </si>
-  <si>
-    <t>soil_ph</t>
-  </si>
-  <si>
-    <t>Soil pH</t>
-  </si>
-  <si>
-    <t>Measure pH of the soil (1 decimal precision).</t>
-  </si>
-  <si>
-    <t>6.4</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t>climate_info</t>
-  </si>
-  <si>
-    <t>Climate Data (auto-filled later)</t>
-  </si>
-  <si>
-    <t>This field will be completed automatically in the web app.</t>
-  </si>
-  <si>
-    <t>group_ga0dq77</t>
-  </si>
-  <si>
-    <t>Section 4 – Sampling Details</t>
-  </si>
-  <si>
-    <t>integer</t>
-  </si>
-  <si>
-    <t>depth_cm</t>
-  </si>
-  <si>
-    <t>Sampling Depth (cm)</t>
-  </si>
-  <si>
-    <t>Enter depth in centimeters.</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>num_samples</t>
-  </si>
-  <si>
-    <t>Number of sub-samples</t>
-  </si>
-  <si>
-    <t>Number of sub-samples collected at this site.</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>tube_id</t>
-  </si>
-  <si>
-    <t>Tube ID</t>
-  </si>
-  <si>
-    <t>Label each physical tube with a unique code using this format: SMP-[sample_id]-[subnumber]-[initials] Example: SMP-COL-2025-001-01-PS Use waterproof labels and indelible ink.</t>
-  </si>
-  <si>
-    <t>SMP-COL-2025-001-01-PS</t>
-  </si>
-  <si>
-    <t>image</t>
-  </si>
-  <si>
-    <t>photo_sample</t>
-  </si>
-  <si>
-    <t>Sample Photo</t>
-  </si>
-  <si>
-    <t>Optional photo of the sample or environment.</t>
-  </si>
-  <si>
-    <t>max-pixels=1024</t>
-  </si>
-  <si>
-    <t>calculate</t>
-  </si>
-  <si>
-    <t>instance_uuid</t>
-  </si>
-  <si>
-    <t>uuid()</t>
-  </si>
-  <si>
-    <t>list_name</t>
-  </si>
-  <si>
-    <t>iq6nb08</t>
-  </si>
-  <si>
-    <t>worm_lab</t>
-  </si>
-  <si>
-    <t>worm~lab</t>
-  </si>
-  <si>
-    <t>sanger_institute</t>
-  </si>
-  <si>
-    <t>Sanger Institute</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>cl7yy10</t>
-  </si>
-  <si>
-    <t>option_1</t>
-  </si>
-  <si>
-    <t>Option 1</t>
-  </si>
-  <si>
-    <t>option_2</t>
-  </si>
-  <si>
-    <t>Option 2</t>
-  </si>
-  <si>
-    <t>option_3</t>
-  </si>
-  <si>
-    <t>Option 3</t>
-  </si>
-  <si>
-    <t>ic4vv27</t>
-  </si>
-  <si>
-    <t>pt7uh58</t>
-  </si>
-  <si>
-    <t>id_string</t>
-  </si>
-  <si>
-    <t>style</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>default_language</t>
-  </si>
-  <si>
-    <t>wwm_soil_sampling</t>
-  </si>
-  <si>
-    <t>v1</t>
-  </si>
-  <si>
-    <t>English (en) (english (en))</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -451,13 +48,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -746,8 +410,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1194,115 +862,120 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>what3words</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>What3Words address</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Optional. Enter the three words for this sampling site, for example filled.count.soap or ///filled.count.soap.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>filled.count.soap</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>regex(., "^(///)?[A-Za-zÀ-ÖØ-öø-ÿ-]+[. ][A-Za-zÀ-ÖØ-öø-ÿ-]+[. ][A-Za-zÀ-ÖØ-öø-ÿ-]+$")</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>group_jy8zq69</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Section 3 – Environmental &amp; Soil Data</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>false</t>
+          <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>select_one habitat_type_list</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>habitat_type</t>
+          <t>group_jy8zq69</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Habitat type</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Select habitat (forest, agricultural, desert, grassland, etc.)</t>
+          <t>Section 3 – Environmental &amp; Soil Data</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Agricultural field</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>select_one soil_type_list</t>
+          <t>select_one habitat_type_list</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>soil_type</t>
+          <t>habitat_type</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Soil type</t>
+          <t>Habitat type</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Choose soil texture (sandy, clay, loamy, etc.)</t>
+          <t>Select habitat (forest, agricultural, desert, grassland, etc.)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sandy loam</t>
+          <t>Agricultural field</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>select_one soil_type_list</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>soil_ph</t>
+          <t>soil_type</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Soil pH</t>
+          <t>Soil type</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Measure pH of the soil (1 decimal precision).</t>
+          <t>Choose soil texture (sandy, clay, loamy, etc.)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1312,95 +985,95 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>Sandy loam</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>climate_info</t>
+          <t>soil_ph</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Climate Data (auto-filled later)</t>
+          <t>Soil pH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>This field will be completed automatically in the web app.</t>
+          <t>Measure pH of the soil (1 decimal precision).</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>6.4</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>climate_info</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Climate Data (auto-filled later)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>This field will be completed automatically in the web app.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>group_ga0dq77</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Section 4 – Sampling Details</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>false</t>
+          <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>depth_cm</t>
+          <t>group_ga0dq77</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sampling Depth (cm)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Enter depth in centimeters.</t>
+          <t>Section 4 – Sampling Details</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>false</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>3</t>
         </is>
       </c>
     </row>
@@ -1412,49 +1085,49 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>num_samples</t>
+          <t>depth_cm</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Number of sub-samples</t>
+          <t>Sampling Depth (cm)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Number of sub-samples collected at this site.</t>
+          <t>Enter depth in centimeters.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tube_id</t>
+          <t>num_samples</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tube ID</t>
+          <t>Number of sub-samples</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Label each physical tube with a unique code using this format: SMP-[sample_id]-[subnumber]-[initials] Example: SMP-COL-2025-001-01-PS Use waterproof labels and indelible ink.</t>
+          <t>Number of sub-samples collected at this site.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1464,66 +1137,98 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SMP-COL-2025-001-01-PS</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>photo_sample</t>
+          <t>tube_id</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sample Photo</t>
+          <t>Tube ID</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Optional photo of the sample or environment.</t>
+          <t>Label each physical tube with a unique code using this format: SMP-[sample_id]-[subnumber]-[initials] Example: SMP-COL-2025-001-01-PS Use waterproof labels and indelible ink.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>max-pixels=1024</t>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SMP-COL-2025-001-01-PS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>photo_sample</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Sample Photo</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Optional photo of the sample or environment.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>max-pixels=1024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>instance_uuid</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>uuid()</t>
         </is>
@@ -1536,8 +1241,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C279"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6288,33 +5997,51 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" t="s">
-        <v>132</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id_string</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>style</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>default_language</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wwm_soil_sampling</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>English (en) (english (en))</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>